<commit_message>
Daily slate 2026-06-29 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-27.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-27.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="E4" t="n">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="F4" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="G4" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="5">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="E7" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F7" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G7" t="n">
-        <v>51.4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1276</v>
+        <v>1356</v>
       </c>
       <c r="E11" t="n">
-        <v>819</v>
+        <v>868</v>
       </c>
       <c r="F11" t="n">
-        <v>457</v>
+        <v>488</v>
       </c>
       <c r="G11" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>797</v>
+        <v>805</v>
       </c>
       <c r="E12" t="n">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="F12" t="n">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G12" t="n">
-        <v>38.3</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="13">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>404</v>
+        <v>422</v>
       </c>
       <c r="E14" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F14" t="n">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="G14" t="n">
-        <v>22.3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>740</v>
+        <v>760</v>
       </c>
       <c r="E15" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F15" t="n">
-        <v>625</v>
+        <v>641</v>
       </c>
       <c r="G15" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="16">
@@ -874,13 +874,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1319</v>
+        <v>1327</v>
       </c>
       <c r="E16" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F16" t="n">
-        <v>1181</v>
+        <v>1188</v>
       </c>
       <c r="G16" t="n">
         <v>10.5</v>
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5265</v>
+        <v>5637</v>
       </c>
       <c r="E17" t="n">
-        <v>929</v>
+        <v>979</v>
       </c>
       <c r="F17" t="n">
-        <v>4336</v>
+        <v>4658</v>
       </c>
       <c r="G17" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
     </row>
   </sheetData>
@@ -1489,16 +1489,16 @@
         <v>126</v>
       </c>
       <c r="D7" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
       <c r="E7" t="n">
-        <v>1276</v>
+        <v>1356</v>
       </c>
       <c r="F7" t="n">
-        <v>38.3</v>
+        <v>38.6</v>
       </c>
       <c r="G7" t="n">
-        <v>797</v>
+        <v>805</v>
       </c>
       <c r="H7" t="n">
         <v>50</v>
@@ -1507,28 +1507,28 @@
         <v>22</v>
       </c>
       <c r="J7" t="n">
-        <v>22.3</v>
+        <v>22</v>
       </c>
       <c r="K7" t="n">
-        <v>404</v>
+        <v>422</v>
       </c>
       <c r="L7" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
       <c r="M7" t="n">
-        <v>740</v>
+        <v>760</v>
       </c>
       <c r="N7" t="n">
         <v>10.5</v>
       </c>
       <c r="O7" t="n">
-        <v>1319</v>
+        <v>1327</v>
       </c>
       <c r="P7" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>5265</v>
+        <v>5637</v>
       </c>
       <c r="R7" t="n">
         <v>87.5</v>
@@ -1537,10 +1537,10 @@
         <v>8</v>
       </c>
       <c r="T7" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="U7" t="n">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1564,10 +1564,10 @@
         <v>5</v>
       </c>
       <c r="AD7" t="n">
-        <v>51.4</v>
+        <v>50</v>
       </c>
       <c r="AE7" t="n">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="AF7" t="n">
         <v>54.9</v>

</xml_diff>